<commit_message>
[Test] Add test execution log for Run 1 (TC-001..TC-027)
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="121">
   <si>
     <t xml:space="preserve">Параметри тестового середовища — Спринт 3</t>
   </si>
@@ -187,7 +187,13 @@
     <t xml:space="preserve">28/10/26 00:27</t>
   </si>
   <si>
-    <t xml:space="preserve">Поля паролів не зберігаються</t>
+    <t xml:space="preserve">failed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-006, BUG-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поля паролів не зберігаються, також проблеми з відображенням кирилиці</t>
   </si>
   <si>
     <t xml:space="preserve">TC-004</t>
@@ -238,9 +244,6 @@
     <t xml:space="preserve">28/10/26 01:15</t>
   </si>
   <si>
-    <t xml:space="preserve">failed</t>
-  </si>
-  <si>
     <t xml:space="preserve">BUG-001</t>
   </si>
   <si>
@@ -358,7 +361,10 @@
     <t xml:space="preserve">blocked</t>
   </si>
   <si>
-    <t xml:space="preserve">Причина: demo відхиляє заявку через внутрішній скоринг (insufficient funds for down payment) незалежно від балансу</t>
+    <t xml:space="preserve">система повертає «insufficient funds for down payment» через внутрішній скоринг demo — 
+це стороннє обмеження, не пов'язане з перевіркою межі суми; 
+виконати кейс і порівняти результат з очікуваним неможливо
+Свідомо не ставлю тут статус failed, адже результат тесту не є багом, на мій погляд. Це саме обмеження ресурсу, тому такий статус підходить тут значно краще</t>
   </si>
   <si>
     <t xml:space="preserve">TC-027</t>
@@ -592,84 +598,88 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -928,195 +938,195 @@
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1144,708 +1154,711 @@
   <dimension ref="A1:H35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="55.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="8"/>
+      <c r="D3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="12"/>
-    </row>
-    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="D4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="11"/>
+      <c r="H4" s="13"/>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="8" t="s">
+      <c r="D5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>54</v>
       </c>
+      <c r="G5" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="12"/>
+      <c r="B6" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="11"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="8"/>
+      <c r="B7" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
+      <c r="A8" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="10"/>
-      <c r="H8" s="12"/>
+      <c r="B8" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="8"/>
+      <c r="B9" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="7"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="12"/>
+      <c r="B10" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="11"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="8"/>
+      <c r="B11" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="7"/>
+      <c r="H11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
+      <c r="A12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" s="10"/>
-      <c r="H12" s="12"/>
+      <c r="B12" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="11"/>
+      <c r="H12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" s="13" t="s">
+      <c r="B13" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="C13" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="D13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" s="15" t="s">
         <v>73</v>
       </c>
+      <c r="H13" s="9" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="H14" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>73</v>
-      </c>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="B15" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G15" s="14" t="s">
+      <c r="C15" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="H15" s="8" t="s">
-        <v>73</v>
+      <c r="D15" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="10" t="s">
+      <c r="B16" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" s="10"/>
-      <c r="H16" s="12"/>
+      <c r="C16" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" s="11"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="B17" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G17" s="6"/>
-      <c r="H17" s="8"/>
+      <c r="C17" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="7"/>
+      <c r="H17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="C18" s="10" t="s">
+      <c r="B18" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D18" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="12"/>
+      <c r="C18" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G18" s="11"/>
+      <c r="H18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="6" t="s">
+      <c r="B19" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G19" s="6"/>
-      <c r="H19" s="8"/>
+      <c r="C19" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G19" s="7"/>
+      <c r="H19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G20" s="10"/>
-      <c r="H20" s="12"/>
+      <c r="C20" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" s="11"/>
+      <c r="H20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C21" s="6" t="s">
+      <c r="B21" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G21" s="6"/>
-      <c r="H21" s="8"/>
+      <c r="C21" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G21" s="7"/>
+      <c r="H21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="n">
+      <c r="A22" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="10" t="s">
+      <c r="B22" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="D22" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G22" s="15" t="s">
+      <c r="C22" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="H22" s="12" t="s">
+      <c r="D22" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="16" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="n">
+      <c r="H22" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="48.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="6" t="s">
+      <c r="B23" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G23" s="14" t="s">
+      <c r="C23" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="D23" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="15" t="s">
         <v>99</v>
       </c>
+      <c r="H23" s="9" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="n">
+      <c r="A24" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C24" s="10" t="s">
+      <c r="B24" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D24" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G24" s="10"/>
-      <c r="H24" s="12"/>
+      <c r="C24" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G24" s="11"/>
+      <c r="H24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="n">
+      <c r="A25" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="C25" s="6" t="s">
+      <c r="B25" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="8"/>
+      <c r="C25" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G25" s="7"/>
+      <c r="H25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="n">
+      <c r="A26" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C26" s="10" t="s">
+      <c r="B26" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="D26" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G26" s="10"/>
-      <c r="H26" s="12"/>
+      <c r="C26" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G26" s="11"/>
+      <c r="H26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C27" s="6" t="s">
+      <c r="B27" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G27" s="6"/>
-      <c r="H27" s="8"/>
-    </row>
-    <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="n">
+      <c r="C27" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G27" s="7"/>
+      <c r="H27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="99.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C28" s="10" t="s">
+      <c r="B28" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D28" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E28" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F28" s="16" t="s">
+      <c r="C28" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="G28" s="10"/>
-      <c r="H28" s="12" t="s">
+      <c r="D28" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F28" s="17" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="n">
+      <c r="G28" s="11"/>
+      <c r="H28" s="13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="102.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="G29" s="7"/>
+      <c r="H29" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F29" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="8" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="17" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>117</v>
+      <c r="B34" s="19" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="B35" s="18" t="s">
+      <c r="A35" s="20" t="s">
         <v>119</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>